<commit_message>
sample_data: drop Utile di esercizio, add DTA, auto-plug Cassa (<5)
Corrections requested:
- Remove "Utile di esercizio" from Tier 1 and Tier 2 (P&L closes into
  Riserve e utili a nuovo at year-end, no separate equity line).
- Tier 2: add "Crediti per imposte anticipate" SP_assets, Y-1=11, Y0=15.

build_sample_data.py now:
- Computes pre/post-plug SP balance for each year.
- Auto-plugs Cassa e disponibilità when |gap| < 5 (rounding tolerance).
- Prints "GAP RESIDUO ... attendo istruzioni" and exits non-zero when
  |gap| >= 5 instead of silently masking the imbalance.

Result:
- Tier 1 / Y0: balanced (sum = 0).
- Tier 2 / Y-1: gap -35 (>= 5) — plug NOT applied, awaiting instructions.
- Tier 2 / Y0:  gap -37 (>= 5) — plug NOT applied, awaiting instructions.

tier2_industrial_clean.xlsx is therefore committed as-is (unbalanced)
pending user decision on the closing approach.

https://claude.ai/code/session_01NBSvkpKwm8FK7SzrAxk78f
</commit_message>
<xml_diff>
--- a/projection_library_kernel_v1.1/projection_library/sample_data/tier1_minimal_balance.xlsx
+++ b/projection_library_kernel_v1.1/projection_library/sample_data/tier1_minimal_balance.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -673,21 +673,6 @@
         <v>-1015</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Utile di esercizio</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>SP_equity</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>-265</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>